<commit_message>
Add sales data and update Excel workbooks
Added a new Sales data.xlsx workbook and updated the existing Excel practice files for the combined task sheet and the IF/IFS/AND/OR exercises. These changes refresh the sample data and workbook content used for formula and task-based Excel practice.
</commit_message>
<xml_diff>
--- a/All in one Task.xlsx
+++ b/All in one Task.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prabh\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3a069205656c65a3/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{964BF48B-2C13-4E61-BD07-B07E2E5E40D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EC960F5B-F609-4DCC-9027-4699E81F7F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7828750-325A-4FA9-B159-480874945AB2}"/>
   </bookViews>
@@ -30,9 +30,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -1098,7 +1095,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E65F43A-176E-4BEE-B2D3-0059C149D9E6}">
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="15.88671875" customWidth="1"/>
@@ -1114,7 +1111,7 @@
     <col min="13" max="13" width="100.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="16.05" customHeight="1">
+    <row r="1" spans="1:14" ht="16.05" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1149,7 +1146,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:14">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -1181,8 +1178,12 @@
       <c r="M2" s="5" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="3" spans="1:13">
+      <c r="N2">
+        <f>_xlfn.XLOOKUP("E103", A2:A11, D2:D11)</f>
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
@@ -1213,7 +1214,7 @@
       <c r="J3" s="1"/>
       <c r="M3" s="5"/>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:14">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1245,8 +1246,12 @@
       <c r="M4" s="5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="5" spans="1:13">
+      <c r="N4">
+        <f>_xlfn.XLOOKUP("E105", A2:A11, E2:E11)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
@@ -1277,7 +1282,7 @@
       <c r="J5" s="1"/>
       <c r="M5" s="5"/>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:14">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -1310,7 +1315,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:14">
       <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
@@ -1341,7 +1346,7 @@
       <c r="J7" s="1"/>
       <c r="M7" s="5"/>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:14">
       <c r="A8" s="2" t="s">
         <v>34</v>
       </c>
@@ -1374,7 +1379,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:14">
       <c r="A9" s="2" t="s">
         <v>36</v>
       </c>
@@ -1405,7 +1410,7 @@
       <c r="J9" s="1"/>
       <c r="M9" s="5"/>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:14">
       <c r="A10" s="2" t="s">
         <v>38</v>
       </c>
@@ -1437,8 +1442,12 @@
       <c r="M10" s="5" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="11" spans="1:13">
+      <c r="N10" t="str">
+        <f>_xlfn.XLOOKUP("E109", A2:A11, B2:B11)</f>
+        <v>Karthik</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" s="2" t="s">
         <v>40</v>
       </c>
@@ -1469,119 +1478,151 @@
       <c r="J11" s="1"/>
       <c r="M11" s="5"/>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:14">
       <c r="M12" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="13" spans="1:13">
+      <c r="N12">
+        <f>_xlfn.XLOOKUP("E107", A2:A11, G2:G11)</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
       <c r="M13" s="5"/>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:14">
       <c r="M14" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:14">
       <c r="M15" s="5"/>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:14">
       <c r="M16" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="13:13">
+    <row r="17" spans="13:14">
       <c r="M17" s="5"/>
     </row>
-    <row r="18" spans="13:13">
+    <row r="18" spans="13:14">
       <c r="M18" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="19" spans="13:13">
+      <c r="N18">
+        <f>_xlfn.XLOOKUP("Sneha", B2:B11, D2:D11)</f>
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="19" spans="13:14">
       <c r="M19" s="5"/>
     </row>
-    <row r="20" spans="13:13">
+    <row r="20" spans="13:14">
       <c r="M20" s="5" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="21" spans="13:13">
+      <c r="N20">
+        <f>_xlfn.XLOOKUP("Ravi", B2:B11, E2:E11)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="13:14">
       <c r="M21" s="5"/>
     </row>
-    <row r="22" spans="13:13">
+    <row r="22" spans="13:14">
       <c r="M22" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="13:13">
+    <row r="23" spans="13:14">
       <c r="M23" s="5"/>
     </row>
-    <row r="24" spans="13:13">
+    <row r="24" spans="13:14">
       <c r="M24" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="13:13">
+    <row r="25" spans="13:14">
       <c r="M25" s="5"/>
     </row>
-    <row r="26" spans="13:13">
+    <row r="26" spans="13:14">
       <c r="M26" s="5" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="27" spans="13:13">
+      <c r="N26">
+        <f>_xlfn.XLOOKUP("Arjun", B2:B11, F2:F11)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="13:14">
       <c r="M27" s="5"/>
     </row>
-    <row r="28" spans="13:13">
+    <row r="28" spans="13:14">
       <c r="M28" s="5" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="29" spans="13:13">
+      <c r="N28">
+        <f>_xlfn.XLOOKUP("E110", A2:A11, D2:D11)</f>
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="29" spans="13:14">
       <c r="M29" s="5"/>
     </row>
-    <row r="30" spans="13:13">
+    <row r="30" spans="13:14">
       <c r="M30" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="13:13">
+    <row r="31" spans="13:14">
       <c r="M31" s="5"/>
     </row>
-    <row r="32" spans="13:13">
+    <row r="32" spans="13:14">
       <c r="M32" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="13:13">
+    <row r="33" spans="13:14">
       <c r="M33" s="5"/>
     </row>
-    <row r="34" spans="13:13">
+    <row r="34" spans="13:14">
       <c r="M34" s="5" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="35" spans="13:13">
+      <c r="N34" t="str">
+        <f>_xlfn.XLOOKUP("E108", A2:A11, C2:C11)</f>
+        <v>SQL</v>
+      </c>
+    </row>
+    <row r="35" spans="13:14">
       <c r="M35" s="5"/>
     </row>
-    <row r="36" spans="13:13">
+    <row r="36" spans="13:14">
       <c r="M36" s="5" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="37" spans="13:13">
+      <c r="N36" t="str">
+        <f>_xlfn.XLOOKUP("Karthik", B2:B11, I2:I11)</f>
+        <v>Excited</v>
+      </c>
+    </row>
+    <row r="37" spans="13:14">
       <c r="M37" s="5"/>
     </row>
-    <row r="38" spans="13:13">
+    <row r="38" spans="13:14">
       <c r="M38" s="5" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="39" spans="13:13">
+      <c r="N38" t="str">
+        <f>_xlfn.XLOOKUP("E104", A2:A11, B2:B11)</f>
+        <v>Anu</v>
+      </c>
+    </row>
+    <row r="39" spans="13:14">
       <c r="M39" s="5"/>
     </row>
-    <row r="40" spans="13:13">
+    <row r="40" spans="13:14">
       <c r="M40" s="5" t="s">
         <v>63</v>
       </c>

</xml_diff>